<commit_message>
Update Nimoloo read-only metrics and Excel report
</commit_message>
<xml_diff>
--- a/public/nimoloo/reports/latest.xlsx
+++ b/public/nimoloo/reports/latest.xlsx
@@ -98,7 +98,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-23T23:55:18Z</t>
+          <t xml:space="preserve">2026-10-23T23:58:22Z</t>
         </is>
       </c>
     </row>
@@ -122,7 +122,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Awaiting verified YouTube API sync</t>
+          <t xml:space="preserve">Waiting for verified existing Nimoloo YouTube channel ID</t>
         </is>
       </c>
     </row>
@@ -313,14 +313,9 @@
           <t xml:space="preserve">Nimoloo Kids</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UCRY6p6rLZkco7tkPiiQ_qeQ</t>
-        </is>
-      </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Awaiting verified YouTube API sync</t>
+          <t xml:space="preserve">Waiting for verified existing Nimoloo YouTube channel ID</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -337,7 +332,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Awaiting verified YouTube API sync</t>
+          <t xml:space="preserve">Waiting for verified existing Nimoloo YouTube channel ID</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -593,20 +588,42 @@
     <row r="6" ht="23" customHeight="1">
       <c r="A6" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nimoloo channel ID not verified</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Previously saved ID failed the official YouTube RSS request (HTTP 404). Removed the unverified channel ID to prevent wrong-channel statistics. A verified ID must come from the existing signed-in YouTube account; do not create a new channel.</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">channel_id_unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="23" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">medium</t>
         </is>
       </c>
-      <c r="B6" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public YouTube refresh incomplete</t>
-        </is>
-      </c>
-      <c r="C6" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nimoloo Kids: YouTube HTTP 404</t>
-        </is>
-      </c>
-      <c r="D6" s="0" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">View counters require API authorization</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatic RSS sync checks public video titles only. For views and subscribers add a YouTube Data API key as a GitHub Actions repository secret, or connect from the web dashboard. Private uploads require OAuth in Termux.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">youtube_public_sync</t>
         </is>
@@ -644,7 +661,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-23T23:55:18Z</t>
+          <t xml:space="preserve">2026-10-23T23:58:22Z</t>
         </is>
       </c>
     </row>
@@ -668,7 +685,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Awaiting verified YouTube API sync</t>
+          <t xml:space="preserve">Waiting for verified existing Nimoloo YouTube channel ID</t>
         </is>
       </c>
     </row>

</xml_diff>